<commit_message>
Give the new DORIS ODK rows WHO order numbers and age groups
The generated rows copy ND01's column layout, which includes WHO's order
and agegroup columns, but the 19 added questions left both empty, so a
form developer could not tell where a row sits or which age group it is
for. Age group is now set on each question in the extension (the web
instrument carries it too) and the generator copies it; a question
without one fails the build. Order numbers extend the anchor's WHO number
with a decimal (30.1, 418.1, 479.1) instead of renumbering, so every
existing WHO order stays valid in the deployed workbooks.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/kb/WHO_VA_2022_Docs/odk-doris-support-rows.xlsx
+++ b/docs/kb/WHO_VA_2022_Docs/odk-doris-support-rows.xlsx
@@ -526,6 +526,11 @@
       </c>
     </row>
     <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>30.1</t>
+        </is>
+      </c>
       <c r="B2" t="inlineStr">
         <is>
           <t>select_one dob_precision</t>
@@ -541,6 +546,11 @@
           <t>selected(${Id10020}, 'no') or selected(${Id10020}, 'ref')</t>
         </is>
       </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
       <c r="F2" t="inlineStr">
         <is>
           <t>Is the month and year, or only the year, of birth known?</t>
@@ -548,6 +558,11 @@
       </c>
     </row>
     <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>30.2</t>
+        </is>
+      </c>
       <c r="B3" t="inlineStr">
         <is>
           <t>date</t>
@@ -563,6 +578,11 @@
           <t>selected(${dob_precision}, 'month_year')</t>
         </is>
       </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
       <c r="F3" t="inlineStr">
         <is>
           <t>In which month and year was the deceased born?</t>
@@ -585,6 +605,11 @@
       </c>
     </row>
     <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>30.3</t>
+        </is>
+      </c>
       <c r="B4" t="inlineStr">
         <is>
           <t>date</t>
@@ -598,6 +623,11 @@
       <c r="D4" t="inlineStr">
         <is>
           <t>selected(${dob_precision}, 'year')</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>ALL</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -680,6 +710,11 @@
       </c>
     </row>
     <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>418.1</t>
+        </is>
+      </c>
       <c r="B6" t="inlineStr">
         <is>
           <t>acknowledge</t>
@@ -695,6 +730,11 @@
           <t>${Id10366} &lt; 500 or ${Id10366} &gt; 6000</t>
         </is>
       </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>N_C</t>
+        </is>
+      </c>
       <c r="F6" t="inlineStr">
         <is>
           <t>A birth weight of ${Id10366} g is unusual. Check the card and confirm the weight is in grammes.</t>
@@ -707,6 +747,11 @@
       </c>
     </row>
     <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>104.1</t>
+        </is>
+      </c>
       <c r="B7" t="inlineStr">
         <is>
           <t>integer</t>
@@ -722,6 +767,11 @@
           <t>selected(${isNeonatal}, '1') and selected(${Id10020}, 'yes') and selected(${Id10022}, 'yes') and ${ageInDays} = 0 and not(selected(${Id10114}, 'yes'))</t>
         </is>
       </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="F7" t="inlineStr">
         <is>
           <t>For how many hours did the baby live?</t>
@@ -739,6 +789,11 @@
       </c>
     </row>
     <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>422.1</t>
+        </is>
+      </c>
       <c r="B8" t="inlineStr">
         <is>
           <t>integer</t>
@@ -754,6 +809,11 @@
           <t>selected(${isNeonatal}, '1') or (selected(${isChild}, '1') and ${ageInMonthsByYear}&lt;12)</t>
         </is>
       </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>N_C</t>
+        </is>
+      </c>
       <c r="F8" t="inlineStr">
         <is>
           <t>How many completed weeks long was the pregnancy? (only if known, e.g. from an antenatal card)</t>
@@ -771,6 +831,11 @@
       </c>
     </row>
     <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>414.1</t>
+        </is>
+      </c>
       <c r="B9" t="inlineStr">
         <is>
           <t>integer</t>
@@ -786,6 +851,11 @@
           <t>selected(${isNeonatal}, '1') or (selected(${isChild}, '1') and ${ageInMonthsByYear}&lt;12)</t>
         </is>
       </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>N_C</t>
+        </is>
+      </c>
       <c r="F9" t="inlineStr">
         <is>
           <t>How old was the baby's mother, in completed years, when the baby was born?</t>
@@ -803,6 +873,11 @@
       </c>
     </row>
     <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>139.1</t>
+        </is>
+      </c>
       <c r="B10" t="inlineStr">
         <is>
           <t>select_one injury_date_known</t>
@@ -818,6 +893,11 @@
           <t>selected(${Id10077}, 'yes')</t>
         </is>
       </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
       <c r="F10" t="inlineStr">
         <is>
           <t>Is the date of the injury known?</t>
@@ -825,6 +905,11 @@
       </c>
     </row>
     <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>139.2</t>
+        </is>
+      </c>
       <c r="B11" t="inlineStr">
         <is>
           <t>date</t>
@@ -840,6 +925,11 @@
           <t>selected(${doris_injury_date_known}, 'full')</t>
         </is>
       </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
       <c r="F11" t="inlineStr">
         <is>
           <t>On what date was (s)he injured?</t>
@@ -862,6 +952,11 @@
       </c>
     </row>
     <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>139.3</t>
+        </is>
+      </c>
       <c r="B12" t="inlineStr">
         <is>
           <t>date</t>
@@ -877,6 +972,11 @@
           <t>selected(${doris_injury_date_known}, 'month_year')</t>
         </is>
       </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
       <c r="F12" t="inlineStr">
         <is>
           <t>In which month and year was (s)he injured?</t>
@@ -899,6 +999,11 @@
       </c>
     </row>
     <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>139.4</t>
+        </is>
+      </c>
       <c r="B13" t="inlineStr">
         <is>
           <t>select_one injury_place</t>
@@ -914,6 +1019,11 @@
           <t>selected(${Id10077}, 'yes')</t>
         </is>
       </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
       <c r="F13" t="inlineStr">
         <is>
           <t>Where did the injury happen?</t>
@@ -921,6 +1031,11 @@
       </c>
     </row>
     <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>139.5</t>
+        </is>
+      </c>
       <c r="B14" t="inlineStr">
         <is>
           <t>select_one legal_war</t>
@@ -936,6 +1051,11 @@
           <t>selected(${Id10077}, 'yes')</t>
         </is>
       </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
       <c r="F14" t="inlineStr">
         <is>
           <t>Was the injury from police or legal action, or from war?</t>
@@ -943,6 +1063,11 @@
       </c>
     </row>
     <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>479.1</t>
+        </is>
+      </c>
       <c r="B15" t="inlineStr">
         <is>
           <t>select_one YES_NO_DK_REF</t>
@@ -958,6 +1083,11 @@
           <t>not(selected(${Id10114}, 'yes'))</t>
         </is>
       </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
       <c r="F15" t="inlineStr">
         <is>
           <t>Did (s)he have an operation before death?</t>
@@ -965,6 +1095,11 @@
       </c>
     </row>
     <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>479.2</t>
+        </is>
+      </c>
       <c r="B16" t="inlineStr">
         <is>
           <t>integer</t>
@@ -980,6 +1115,11 @@
           <t>selected(${doris_surgery_performed}, 'yes')</t>
         </is>
       </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
       <c r="F16" t="inlineStr">
         <is>
           <t>How long before death was the operation? (number)</t>
@@ -997,6 +1137,11 @@
       </c>
     </row>
     <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>479.3</t>
+        </is>
+      </c>
       <c r="B17" t="inlineStr">
         <is>
           <t>select_one time_unit</t>
@@ -1012,6 +1157,11 @@
           <t>selected(${doris_surgery_performed}, 'yes') and ${doris_surgery_when} != 88 and ${doris_surgery_when} != 99</t>
         </is>
       </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
       <c r="F17" t="inlineStr">
         <is>
           <t>Unit</t>
@@ -1019,6 +1169,11 @@
       </c>
     </row>
     <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>479.4</t>
+        </is>
+      </c>
       <c r="B18" t="inlineStr">
         <is>
           <t>text</t>
@@ -1034,6 +1189,11 @@
           <t>selected(${doris_surgery_performed}, 'yes')</t>
         </is>
       </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
       <c r="F18" t="inlineStr">
         <is>
           <t>What operation was done?</t>
@@ -1041,6 +1201,11 @@
       </c>
     </row>
     <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>479.5</t>
+        </is>
+      </c>
       <c r="B19" t="inlineStr">
         <is>
           <t>text</t>
@@ -1056,6 +1221,11 @@
           <t>selected(${doris_surgery_performed}, 'yes')</t>
         </is>
       </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
       <c r="F19" t="inlineStr">
         <is>
           <t>For what illness or condition was it done?</t>
@@ -1063,6 +1233,11 @@
       </c>
     </row>
     <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>503.1</t>
+        </is>
+      </c>
       <c r="B20" t="inlineStr">
         <is>
           <t>select_one YES_NO_DK_REF</t>
@@ -1073,6 +1248,11 @@
           <t>doris_autopsy_requested</t>
         </is>
       </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
       <c r="F20" t="inlineStr">
         <is>
           <t>Was an autopsy (post-mortem examination) requested?</t>
@@ -1080,6 +1260,11 @@
       </c>
     </row>
     <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>503.2</t>
+        </is>
+      </c>
       <c r="B21" t="inlineStr">
         <is>
           <t>select_one YES_NO_DK_REF</t>
@@ -1093,6 +1278,11 @@
       <c r="D21" t="inlineStr">
         <is>
           <t>selected(${doris_autopsy_requested}, 'yes')</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>ALL</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -1950,7 +2140,7 @@
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>ND01 row numbers are those of the unmodified workbook: apply the blocks bottom-up (A8, A7, A4, A2, A5, A10, A9, A6, A3, A1) so the numbers stay valid. Add the choices at the end of the choices sheet. Hindi and other label columns follow each workbook's languages. Bump settings.version before deploying.</t>
+          <t>ND01 row numbers are those of the unmodified workbook: apply the blocks bottom-up (A8, A7, A4, A2, A5, A10, A9, A6, A3, A1) so the numbers stay valid. Add the choices at the end of the choices sheet. An added row's order is its ND01 anchor's order plus .1, .2... (text, so WHO's orders stay unchanged). Hindi and other label columns follow each workbook's languages. Bump settings.version before deploying.</t>
         </is>
       </c>
     </row>

</xml_diff>